<commit_message>
chore: sync Guru-WorkSpace (DeepEval, AITesterBlueprint3x update, social_ai_agent content)
</commit_message>
<xml_diff>
--- a/Guru-WorkSpace/social_ai_agent/content.xlsx
+++ b/Guru-WorkSpace/social_ai_agent/content.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="24">
   <si>
     <t>Date</t>
   </si>
@@ -105,60 +105,119 @@
     <t>"Mastering Audience Segmentation: A Comprehensive Guide for HCL Unica Users"</t>
   </si>
   <si>
-    <t xml:space="preserve">Title: Mastering Audience Segmentation: A Comprehensive Guide for HCL Unica Users 🔎
-Hello, fellow HCL Unica enthusiasts! 🖥️
-I'm thrilled to share a valuable resource that's bound to elevate your marketing game – our comprehensive guide on Mastering Audience Segmentation. This guide is tailored specifically for HCL Unica users like us, who understand the power of data-driven marketing.
-Segementing your audience is no longer a nice-to-have—it's a must-have in today's complex marketing landscape. With HCL Unica, we have the tools to make it easier than ever. But knowing how to wield these tools effectively can be the difference between a mediocre campaign and a game-changing one.
-Our guide dives deep into the art and science of audience segmentation. You'll learn:
-1. The importance of understanding your audience – and how to do it effectively with HCL Unica's data analytics capabilities.
-2. Strategies for creating meaningful, actionable audience segments – turning raw data into insights that drive results.
-3. Tips for optimizing your segments for maximum engagement – ensuring your messages resonate with your audience.
-4. Case studies showcasing successful audience segmentation strategies – learn from the best and apply these lessons to your own campaigns.
-Remember, audience segmentation is not just about categorizing people – it's about understanding them. By mastering this art, we can create more personalized, effective, and meaningful marketing experiences.
-So, grab your copy of the guide – and let's take our HCL Unica skills to the next level! 🚀
-#StayCurious #DataDrivenMarketing #HCLUnica #AudienceSegmentation #MarketingTips</t>
+    <t xml:space="preserve">In an era where customer expectations are skyrocketing faster than the Milky Way's expanding galaxies—enter HCL Unica, a trailblazer redefining customer engagement.
+Dive deep into their customer journey orchestration strategy, and you'll find a symphony of seamless, personalized interactions—a ballet of brand-consumer exchanges that leaves both parties enchanted.
+Unica's approach is a breath of fresh air in the digital marketing landscape—it's not just about selling products; it's about crafting experiences. They've mastered the art of weaving together disparate touchpoints—from emails to social media, web experiences, and beyond—creating a harmonious narrative that resonates with customers at every turn.
+Their secret sauce? Advanced AI and machine learning, which predict customer behavior with uncanny accuracy—anticipating needs before they're even articulated. This proactive approach is a game-changer, setting Unica apart from the pack.
+But it's not just about being smart—it's about being sensitive. Unica understands that each customer is unique, with their own preferences, pain points, and passions. So they tailor experiences to reflect these individualities, fostering a connection that transcends mere transactions.
+In a world where customer loyalty is as elusive as the Holy Grail—HCL Unica's customer journey orchestration strategy is the beacon guiding businesses towards a brighter future. So, join the revolution—let's reimagine customer engagement together, with HCL Unica leading the way.</t>
   </si>
   <si>
     <t xml:space="preserve">1.
-HEADLINE: Welcome to Mastering Audience Segmentation
-BODY: Dive into our comprehensive guide designed specifically for HCL Unica users.
-CAPTION: Start your journey to better audience segmentation today!
+HEADLINE: Welcome to the Revolution! |
+BODY: Explore how HCL Unica is transforming customer engagement with its cutting-edge Customer Journey Orchestration strategy. |
+CAPTION: Join us as we navigate the future of customer interaction!
 2.
-HEADLINE: Understanding Audience Segmentation
-BODY: Learn how audience segmentation can improve your marketing strategies and campaign performance.
-CAPTION: Segmentation is key to reaching the right audience at the right time!
+HEADLINE: Customer Journey Orchestration |
+BODY: A seamless, personalized, and unified approach to understanding and optimizing every customer touchpoint. |
+CAPTION: Discover the power of a customer journey that adapts to your unique needs!
 3.
-HEADLINE: The Power of HCL Unica
-BODY: Discover how HCL Unica streamlines audience segmentation and boosts marketing effectiveness.
-CAPTION: HCL Unica is your one-stop solution for seamless segmentation!
+HEADLINE: The Power of Data Integration |
+BODY: Harness the full potential of your customer data through our robust integration capabilities. |
+CAPTION: Say goodbye to siloed data and hello to a holistic understanding of your customers!
 4.
-HEADLINE: The Basics of Audience Segmentation
-BODY: Explore the fundamentals of audience segmentation, including demographics, behaviors, and preferences.
-CAPTION: Lay a strong foundation for effective audience segmentation!
+HEADLINE: Real-Time Analytics and Insights |
+BODY: Make informed decisions with real-time insights into customer behavior and preferences. |
+CAPTION: Stay ahead of the curve with actionable insights at your fingertips!
 5.
-HEADLINE: Advanced Segmentation Techniques
-BODY: Delve into advanced techniques like propensity modeling and predictive analytics.
-CAPTION: Take your audience segmentation to the next level!
+HEADLINE: Personalized, Seamless Experiences |
+BODY: Deliver personalized and consistent experiences across all channels, driving customer loyalty and satisfaction. |
+CAPTION: Experience the difference a unified customer journey can make!
 6.
-HEADLINE: Data-Driven Segmentation
-BODY: Understand the importance of using data-driven methods to create more accurate and valuable audience segments.
-CAPTION: Let your data drive your audience segmentation strategies!
+HEADLINE: Scalable and Adaptable |
+BODY: Our solution grows with your business, adapting to your evolving customer needs and expectations. |
+CAPTION: Empower your business to adapt and thrive in an ever-changing market!
 7.
-HEADLINE: Personalized Marketing Campaigns
-BODY: Learn how to use audience segmentation to create highly personalized marketing campaigns that convert.
-CAPTION: Tailor your campaigns for maximum impact and ROI!
+HEADLINE: Proven Results |
+BODY: Learn about the success stories of businesses that have revolutionized their customer engagement with HCL Unica. |
+CAPTION: Discover the impact a customer-centric approach can have on your bottom line!
 8.
-HEADLINE: Measuring Segmentation Success
-BODY: Discover key metrics for measuring the success of your audience segmentation efforts.
-CAPTION: Measure your success and continuously improve your strategies!
+HEADLINE: The Future of Customer Engagement |
+BODY: Prepare for the future with HCL Unica's forward-thinking approach to customer journey orchestration. |
+CAPTION: Join us in shaping the future of customer engagement!
 9.
-HEADLINE: Tips for Effective Segmentation
-BODY: Receive practical tips and best practices for implementing audience segmentation in your marketing efforts.
-CAPTION: Apply these tips to see real results in your audience segmentation!
+HEADLINE: Ready to Revolutionize? |
+BODY: Contact us to learn more about how HCL Unica can transform your customer engagement strategy. |
+CAPTION: Take the first step towards a customer-centric future!
 10.
-HEADLINE: Mastering Audience Segmentation: Next Steps
-BODY: Take the knowledge you've gained and start mastering audience segmentation with HCL Unica today!
-CAPTION: Don't wait – start mastering audience segmentation now!</t>
+HEADLINE: Thank You! |
+BODY: We appreciate you taking the time to learn about HCL Unica's Customer Journey Orchestration strategy. |
+CAPTION: Stay tuned for more insights and updates on our customer-centric solutions!</t>
+  </si>
+  <si>
+    <t>"Revolutionizing Customer Experience: Mastering Real-time Personalization with HCL Unica"</t>
+  </si>
+  <si>
+    <t>"Revolutionizing Customer Engagement: A Deep Dive into HCL Unica's Customer Journey Orchestration Strategy"</t>
+  </si>
+  <si>
+    <t>2026-09-06</t>
+  </si>
+  <si>
+    <t>"Unleashing Personalized Customer Experiences with Unica Interact: A Comprehensive Overview"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">In the dynamic realm of modern marketing, one tool has emerged as a game-changer — Customer Journey Orchestration, powered by HCL Unica.
+An emphatic leap from traditional marketing approaches, this innovative strategy weaves a seamless, personalized narrative throughout a customer's interaction with a brand. It's akin to composing a symphony—each touchpoint, a note, harmonizing to create a captivating and engaging experience.
+HCL Unica, a trailblazer in the field, offers a robust platform that empowers businesses to orchestrate these journeys with precision and finesse. It's not just about sending emails or displaying ads—it's about understanding and anticipating customer needs, and delivering relevant, timely, and compelling content that resonates.
+The power of Customer Journey Orchestration lies in its ability to transform raw data into actionable insights—predicting customer behavior, recommending strategies, and continuously optimizing engagement. It's marketing that's smart, adaptive, and genuinely customer-centric.
+In a world where customer expectations are skyrocketing, HCL Unica provides the orchestral score needed to conduct a symphony of customer experiences—a symphony that's both beautiful to hear and effective in driving business growth.
+Embrace the future of marketing—explore the power of Customer Journey Orchestration with HCL Unica. Let's redefine customer engagement, one harmonious note at a time.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.
+   HEADLINE: Welcome to our Journey! 🚀
+   BODY: Join us as we delve into the transformative world of Customer Journey Orchestration with HCL Unica.
+   CAPTION: Unlock the power of personalized customer experiences.
+2.
+   HEADLINE: What is Customer Journey Orchestration? 🤔
+   BODY: It's the art of creating seamless, personalized, and contextual customer experiences across multiple touchpoints and channels.
+   CAPTION: Say goodbye to fragmented customer journeys.
+3.
+   HEADLINE: The Power of HCL Unica 💥
+   BODY: HCL Unica is a leading Customer Journey Orchestration solution that enables businesses to understand, anticipate, and fulfill customer needs in real-time.
+   CAPTION: Revolutionize your customer interactions.
+4.
+   HEADLINE: Understanding the Customer 🎯
+   BODY: HCL Unica allows businesses to gain a 360-degree view of their customers, understanding their preferences, behavior, and needs.
+   CAPTION: Know your customer better than they know themselves.
+5.
+   HEADLINE: Anticipate Customer Needs 🔮
+   BODY: With advanced AI and machine learning capabilities, HCL Unica predicts customer behavior and delivers personalized, timely, and relevant experiences.
+   CAPTION: Predict their needs before they do.
+6.
+   HEADLINE: Seamless Omnichannel Experiences 🌐
+   BODY: HCL Unica enables businesses to orchestrate customer journeys across multiple channels, providing a consistent and seamless customer experience.
+   CAPTION: One customer, multiple touchpoints.
+7.
+   HEADLINE: Real-time Decision Making ⚡
+   BODY: HCL Unica's real-time decision-making capabilities allow businesses to respond quickly to customer interactions, ensuring that every moment matters.
+   CAPTION: Make every moment count.
+8.
+   HEADLINE: Increase Customer Loyalty 🤝
+   BODY: By delivering personalized and relevant experiences, HCL Unica helps businesses increase customer loyalty and retention.
+   CAPTION: Keep them coming back for more.
+9.
+   HEADLINE: Drive Business Growth 🚀
+   BODY: HCL Unica's customer journey orchestration solutions help businesses drive growth by increasing sales, improving customer satisfaction, and reducing churn.
+   CAPTION: Growth is not just about adding new customers, but retaining the old ones too.
+10.
+   HEADLINE: Let's Explore Together! 🌟
+   BODY: Join us on this journey to understand how HCL Unica can transform your customer interactions and drive business growth.
+   CAPTION: The future of customer engagement is here. Let's shape it together.</t>
+  </si>
+  <si>
+    <t>"Exploring the Power of Customer Journey Orchestration with HCL Unica"</t>
   </si>
 </sst>
 </file>
@@ -538,7 +597,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.2" defaultColWidth="8.83203125"/>
   <cols>
     <col min="1" max="1" width="20" style="1" customWidth="1"/>
@@ -649,6 +708,74 @@
         <v>9</v>
       </c>
     </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>

</xml_diff>